<commit_message>
vault backup: 2026-10-22 17:08:54
</commit_message>
<xml_diff>
--- a/outputs/synopsys-vip-20261022/Synopsys_VIP采购清单_20261022.xlsx
+++ b/outputs/synopsys-vip-20261022/Synopsys_VIP采购清单_20261022.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购目录" sheetId="1" r:id="Ra435f9c701c14bbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购确认" sheetId="2" r:id="R94aa759694bf4c0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购目录" sheetId="1" r:id="Rfecc581c2ac84330"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购确认" sheetId="2" r:id="R5686ca2606eb4e8e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -88,7 +88,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -134,6 +134,18 @@
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -154,9 +166,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VIPCatalog" displayName="VIPCatalog" ref="A7:N84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:N84"/>
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VIPCatalog" displayName="VIPCatalog" ref="A7:P84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:P84"/>
+  <x:tableColumns count="16">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="类别"/>
     <x:tableColumn id="3" name="协议 / 家族"/>
@@ -171,6 +183,8 @@
     <x:tableColumn id="12" name="含 Test Suite"/>
     <x:tableColumn id="13" name="报价金额"/>
     <x:tableColumn id="14" name="币种"/>
+    <x:tableColumn id="15" name="来源说明"/>
+    <x:tableColumn id="16" name="官方来源 URL"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -412,7 +426,7 @@
     <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="11" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="3" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -575,7 +589,9 @@
       <x:c r="N7" s="9" t="str">
         <x:v>币种</x:v>
       </x:c>
-      <x:c r="O7" s="1" t="str"/>
+      <x:c r="O7" s="1" t="str">
+        <x:v>来源说明</x:v>
+      </x:c>
       <x:c r="P7" s="11" t="str">
         <x:v>官方来源 URL</x:v>
       </x:c>
@@ -609,7 +625,9 @@
       <x:c r="L8" s="12" t="str"/>
       <x:c r="M8" s="14"/>
       <x:c r="N8" s="12" t="str"/>
-      <x:c r="O8" s="4" t="str"/>
+      <x:c r="O8" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P8" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/amba/amba-chi.html</x:v>
       </x:c>
@@ -643,7 +661,9 @@
       <x:c r="L9" s="12" t="str"/>
       <x:c r="M9" s="14"/>
       <x:c r="N9" s="12" t="str"/>
-      <x:c r="O9" s="4" t="str"/>
+      <x:c r="O9" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P9" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/amba/amba-axi.html</x:v>
       </x:c>
@@ -677,7 +697,9 @@
       <x:c r="L10" s="12" t="str"/>
       <x:c r="M10" s="14"/>
       <x:c r="N10" s="12" t="str"/>
-      <x:c r="O10" s="4" t="str"/>
+      <x:c r="O10" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P10" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/amba/amba-ace.html</x:v>
       </x:c>
@@ -711,7 +733,9 @@
       <x:c r="L11" s="12" t="str"/>
       <x:c r="M11" s="14"/>
       <x:c r="N11" s="12" t="str"/>
-      <x:c r="O11" s="4" t="str"/>
+      <x:c r="O11" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P11" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/amba/amba-ahb.html</x:v>
       </x:c>
@@ -745,7 +769,9 @@
       <x:c r="L12" s="12" t="str"/>
       <x:c r="M12" s="14"/>
       <x:c r="N12" s="12" t="str"/>
-      <x:c r="O12" s="4" t="str"/>
+      <x:c r="O12" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P12" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/amba/amba-apb.html</x:v>
       </x:c>
@@ -779,7 +805,9 @@
       <x:c r="L13" s="12" t="str"/>
       <x:c r="M13" s="14"/>
       <x:c r="N13" s="12" t="str"/>
-      <x:c r="O13" s="4" t="str"/>
+      <x:c r="O13" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P13" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/amba/amba-atb.html</x:v>
       </x:c>
@@ -813,7 +841,9 @@
       <x:c r="L14" s="12" t="str"/>
       <x:c r="M14" s="14"/>
       <x:c r="N14" s="12" t="str"/>
-      <x:c r="O14" s="4" t="str"/>
+      <x:c r="O14" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P14" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/amba/amba-stream.html</x:v>
       </x:c>
@@ -847,7 +877,9 @@
       <x:c r="L15" s="12" t="str"/>
       <x:c r="M15" s="14"/>
       <x:c r="N15" s="12" t="str"/>
-      <x:c r="O15" s="4" t="str"/>
+      <x:c r="O15" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P15" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/amba/amba-cxs.html</x:v>
       </x:c>
@@ -881,7 +913,9 @@
       <x:c r="L16" s="12" t="str"/>
       <x:c r="M16" s="14"/>
       <x:c r="N16" s="12" t="str"/>
-      <x:c r="O16" s="4" t="str"/>
+      <x:c r="O16" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P16" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/amba/amba-c2c.html</x:v>
       </x:c>
@@ -915,7 +949,9 @@
       <x:c r="L17" s="12" t="str"/>
       <x:c r="M17" s="14"/>
       <x:c r="N17" s="12" t="str"/>
-      <x:c r="O17" s="4" t="str"/>
+      <x:c r="O17" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P17" s="4" t="str">
         <x:v>https://www.synopsys.com/blogs/chip-design/industry-first-verification-ip-arm-amb-dtih.html</x:v>
       </x:c>
@@ -949,7 +985,9 @@
       <x:c r="L18" s="12" t="str"/>
       <x:c r="M18" s="14"/>
       <x:c r="N18" s="12" t="str"/>
-      <x:c r="O18" s="4" t="str"/>
+      <x:c r="O18" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P18" s="4" t="str">
         <x:v>https://www.synopsys.com/zh-cn/verification/verification-ip.html</x:v>
       </x:c>
@@ -983,7 +1021,9 @@
       <x:c r="L19" s="12" t="str"/>
       <x:c r="M19" s="14"/>
       <x:c r="N19" s="12" t="str"/>
-      <x:c r="O19" s="4" t="str"/>
+      <x:c r="O19" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P19" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/TileLink.html</x:v>
       </x:c>
@@ -1017,7 +1057,9 @@
       <x:c r="L20" s="12" t="str"/>
       <x:c r="M20" s="14"/>
       <x:c r="N20" s="12" t="str"/>
-      <x:c r="O20" s="4" t="str"/>
+      <x:c r="O20" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P20" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/ocp.html</x:v>
       </x:c>
@@ -1051,7 +1093,9 @@
       <x:c r="L21" s="12" t="str"/>
       <x:c r="M21" s="14"/>
       <x:c r="N21" s="12" t="str"/>
-      <x:c r="O21" s="4" t="str"/>
+      <x:c r="O21" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P21" s="4" t="str">
         <x:v>https://www.synopsys.com/zh-cn/verification/verification-ip.html</x:v>
       </x:c>
@@ -1085,7 +1129,9 @@
       <x:c r="L22" s="12" t="str"/>
       <x:c r="M22" s="14"/>
       <x:c r="N22" s="12" t="str"/>
-      <x:c r="O22" s="4" t="str"/>
+      <x:c r="O22" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P22" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/ddr5.html</x:v>
       </x:c>
@@ -1119,7 +1165,9 @@
       <x:c r="L23" s="12" t="str"/>
       <x:c r="M23" s="14"/>
       <x:c r="N23" s="12" t="str"/>
-      <x:c r="O23" s="4" t="str"/>
+      <x:c r="O23" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P23" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/ddr5.html</x:v>
       </x:c>
@@ -1153,7 +1201,9 @@
       <x:c r="L24" s="12" t="str"/>
       <x:c r="M24" s="14"/>
       <x:c r="N24" s="12" t="str"/>
-      <x:c r="O24" s="4" t="str"/>
+      <x:c r="O24" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P24" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/ip-lpddr.html</x:v>
       </x:c>
@@ -1187,7 +1237,9 @@
       <x:c r="L25" s="12" t="str"/>
       <x:c r="M25" s="14"/>
       <x:c r="N25" s="12" t="str"/>
-      <x:c r="O25" s="4" t="str"/>
+      <x:c r="O25" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P25" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/hbm-verificationip.html</x:v>
       </x:c>
@@ -1221,7 +1273,9 @@
       <x:c r="L26" s="12" t="str"/>
       <x:c r="M26" s="14"/>
       <x:c r="N26" s="12" t="str"/>
-      <x:c r="O26" s="4" t="str"/>
+      <x:c r="O26" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P26" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/gddr6.html</x:v>
       </x:c>
@@ -1255,7 +1309,9 @@
       <x:c r="L27" s="12" t="str"/>
       <x:c r="M27" s="14"/>
       <x:c r="N27" s="12" t="str"/>
-      <x:c r="O27" s="4" t="str"/>
+      <x:c r="O27" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P27" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/hmc-verification-ip.html</x:v>
       </x:c>
@@ -1289,7 +1345,9 @@
       <x:c r="L28" s="12" t="str"/>
       <x:c r="M28" s="14"/>
       <x:c r="N28" s="12" t="str"/>
-      <x:c r="O28" s="4" t="str"/>
+      <x:c r="O28" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P28" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/dfi-verification-ip.html</x:v>
       </x:c>
@@ -1323,7 +1381,9 @@
       <x:c r="L29" s="12" t="str"/>
       <x:c r="M29" s="14"/>
       <x:c r="N29" s="12" t="str"/>
-      <x:c r="O29" s="4" t="str"/>
+      <x:c r="O29" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P29" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/nvdimm-p.html</x:v>
       </x:c>
@@ -1357,7 +1417,9 @@
       <x:c r="L30" s="12" t="str"/>
       <x:c r="M30" s="14"/>
       <x:c r="N30" s="12" t="str"/>
-      <x:c r="O30" s="4" t="str"/>
+      <x:c r="O30" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P30" s="4" t="str">
         <x:v>https://www.synopsys.com/zh-cn/verification/verification-ip.html</x:v>
       </x:c>
@@ -1391,7 +1453,9 @@
       <x:c r="L31" s="12" t="str"/>
       <x:c r="M31" s="14"/>
       <x:c r="N31" s="12" t="str"/>
-      <x:c r="O31" s="4" t="str"/>
+      <x:c r="O31" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P31" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/emmc-verification-ip.html</x:v>
       </x:c>
@@ -1425,7 +1489,9 @@
       <x:c r="L32" s="12" t="str"/>
       <x:c r="M32" s="14"/>
       <x:c r="N32" s="12" t="str"/>
-      <x:c r="O32" s="4" t="str"/>
+      <x:c r="O32" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P32" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/sd-host-card.html</x:v>
       </x:c>
@@ -1459,7 +1525,9 @@
       <x:c r="L33" s="12" t="str"/>
       <x:c r="M33" s="14"/>
       <x:c r="N33" s="12" t="str"/>
-      <x:c r="O33" s="4" t="str"/>
+      <x:c r="O33" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P33" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/uhs-ii-sd-tran.html</x:v>
       </x:c>
@@ -1493,7 +1561,9 @@
       <x:c r="L34" s="12" t="str"/>
       <x:c r="M34" s="14"/>
       <x:c r="N34" s="12" t="str"/>
-      <x:c r="O34" s="4" t="str"/>
+      <x:c r="O34" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P34" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/onfi.html</x:v>
       </x:c>
@@ -1527,7 +1597,9 @@
       <x:c r="L35" s="12" t="str"/>
       <x:c r="M35" s="14"/>
       <x:c r="N35" s="12" t="str"/>
-      <x:c r="O35" s="4" t="str"/>
+      <x:c r="O35" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P35" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/toggglenand.html</x:v>
       </x:c>
@@ -1561,7 +1633,9 @@
       <x:c r="L36" s="12" t="str"/>
       <x:c r="M36" s="14"/>
       <x:c r="N36" s="12" t="str"/>
-      <x:c r="O36" s="4" t="str"/>
+      <x:c r="O36" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P36" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/memory/spi-qspi.html</x:v>
       </x:c>
@@ -1595,7 +1669,9 @@
       <x:c r="L37" s="12" t="str"/>
       <x:c r="M37" s="14"/>
       <x:c r="N37" s="12" t="str"/>
-      <x:c r="O37" s="4" t="str"/>
+      <x:c r="O37" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P37" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/pcie.html</x:v>
       </x:c>
@@ -1629,7 +1705,9 @@
       <x:c r="L38" s="12" t="str"/>
       <x:c r="M38" s="14"/>
       <x:c r="N38" s="12" t="str"/>
-      <x:c r="O38" s="4" t="str"/>
+      <x:c r="O38" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P38" s="4" t="str">
         <x:v>https://www.synopsys.com/zh-cn/verification/verification-ip.html</x:v>
       </x:c>
@@ -1663,7 +1741,9 @@
       <x:c r="L39" s="12" t="str"/>
       <x:c r="M39" s="14"/>
       <x:c r="N39" s="12" t="str"/>
-      <x:c r="O39" s="4" t="str"/>
+      <x:c r="O39" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P39" s="4" t="str">
         <x:v>https://www.synopsys.com/designware-ip/interface-ip/ccix.html</x:v>
       </x:c>
@@ -1697,7 +1777,9 @@
       <x:c r="L40" s="12" t="str"/>
       <x:c r="M40" s="14"/>
       <x:c r="N40" s="12" t="str"/>
-      <x:c r="O40" s="4" t="str"/>
+      <x:c r="O40" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P40" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/subsystems/compute-express-link.html</x:v>
       </x:c>
@@ -1731,7 +1813,9 @@
       <x:c r="L41" s="12" t="str"/>
       <x:c r="M41" s="14"/>
       <x:c r="N41" s="12" t="str"/>
-      <x:c r="O41" s="4" t="str"/>
+      <x:c r="O41" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P41" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/subsystems/vc-verification-ip-for-ucie.html</x:v>
       </x:c>
@@ -1765,7 +1849,9 @@
       <x:c r="L42" s="12" t="str"/>
       <x:c r="M42" s="14"/>
       <x:c r="N42" s="12" t="str"/>
-      <x:c r="O42" s="4" t="str"/>
+      <x:c r="O42" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P42" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/ualink.html</x:v>
       </x:c>
@@ -1799,7 +1885,9 @@
       <x:c r="L43" s="12" t="str"/>
       <x:c r="M43" s="14"/>
       <x:c r="N43" s="12" t="str"/>
-      <x:c r="O43" s="4" t="str"/>
+      <x:c r="O43" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P43" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/ethernet/ethernet-1-6t.html</x:v>
       </x:c>
@@ -1833,7 +1921,9 @@
       <x:c r="L44" s="12" t="str"/>
       <x:c r="M44" s="14"/>
       <x:c r="N44" s="12" t="str"/>
-      <x:c r="O44" s="4" t="str"/>
+      <x:c r="O44" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P44" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/ethernet/ethernet-avb.html</x:v>
       </x:c>
@@ -1867,7 +1957,9 @@
       <x:c r="L45" s="12" t="str"/>
       <x:c r="M45" s="14"/>
       <x:c r="N45" s="12" t="str"/>
-      <x:c r="O45" s="4" t="str"/>
+      <x:c r="O45" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P45" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/automotive/ethernet.html</x:v>
       </x:c>
@@ -1901,7 +1993,9 @@
       <x:c r="L46" s="12" t="str"/>
       <x:c r="M46" s="14"/>
       <x:c r="N46" s="12" t="str"/>
-      <x:c r="O46" s="4" t="str"/>
+      <x:c r="O46" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P46" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/ethernet/uec.html</x:v>
       </x:c>
@@ -1935,7 +2029,9 @@
       <x:c r="L47" s="12" t="str"/>
       <x:c r="M47" s="14"/>
       <x:c r="N47" s="12" t="str"/>
-      <x:c r="O47" s="4" t="str"/>
+      <x:c r="O47" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P47" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/interlaken.html</x:v>
       </x:c>
@@ -1969,7 +2065,9 @@
       <x:c r="L48" s="12" t="str"/>
       <x:c r="M48" s="14"/>
       <x:c r="N48" s="12" t="str"/>
-      <x:c r="O48" s="4" t="str"/>
+      <x:c r="O48" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P48" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/fibre-channel.html</x:v>
       </x:c>
@@ -2003,7 +2101,9 @@
       <x:c r="L49" s="12" t="str"/>
       <x:c r="M49" s="14"/>
       <x:c r="N49" s="12" t="str"/>
-      <x:c r="O49" s="4" t="str"/>
+      <x:c r="O49" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P49" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/cpri.html</x:v>
       </x:c>
@@ -2037,7 +2137,9 @@
       <x:c r="L50" s="12" t="str"/>
       <x:c r="M50" s="14"/>
       <x:c r="N50" s="12" t="str"/>
-      <x:c r="O50" s="4" t="str"/>
+      <x:c r="O50" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P50" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/subsystems/verification-ip-usb2.html</x:v>
       </x:c>
@@ -2071,7 +2173,9 @@
       <x:c r="L51" s="12" t="str"/>
       <x:c r="M51" s="14"/>
       <x:c r="N51" s="12" t="str"/>
-      <x:c r="O51" s="4" t="str"/>
+      <x:c r="O51" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P51" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/usb/usb.html</x:v>
       </x:c>
@@ -2105,7 +2209,9 @@
       <x:c r="L52" s="12" t="str"/>
       <x:c r="M52" s="14"/>
       <x:c r="N52" s="12" t="str"/>
-      <x:c r="O52" s="4" t="str"/>
+      <x:c r="O52" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P52" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/subsystems/vc-verification-ip-usb4.html</x:v>
       </x:c>
@@ -2139,7 +2245,9 @@
       <x:c r="L53" s="12" t="str"/>
       <x:c r="M53" s="14"/>
       <x:c r="N53" s="12" t="str"/>
-      <x:c r="O53" s="4" t="str"/>
+      <x:c r="O53" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P53" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/usb/usb-power-delivery.html</x:v>
       </x:c>
@@ -2173,7 +2281,9 @@
       <x:c r="L54" s="12" t="str"/>
       <x:c r="M54" s="14"/>
       <x:c r="N54" s="12" t="str"/>
-      <x:c r="O54" s="4" t="str"/>
+      <x:c r="O54" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P54" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/storage/nvme.html</x:v>
       </x:c>
@@ -2207,7 +2317,9 @@
       <x:c r="L55" s="12" t="str"/>
       <x:c r="M55" s="14"/>
       <x:c r="N55" s="12" t="str"/>
-      <x:c r="O55" s="4" t="str"/>
+      <x:c r="O55" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P55" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/storage/sas.html</x:v>
       </x:c>
@@ -2241,7 +2353,9 @@
       <x:c r="L56" s="12" t="str"/>
       <x:c r="M56" s="14"/>
       <x:c r="N56" s="12" t="str"/>
-      <x:c r="O56" s="4" t="str"/>
+      <x:c r="O56" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P56" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/storage/sata.html</x:v>
       </x:c>
@@ -2275,7 +2389,9 @@
       <x:c r="L57" s="12" t="str"/>
       <x:c r="M57" s="14"/>
       <x:c r="N57" s="12" t="str"/>
-      <x:c r="O57" s="4" t="str"/>
+      <x:c r="O57" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P57" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/mipi/ufs.html</x:v>
       </x:c>
@@ -2309,7 +2425,9 @@
       <x:c r="L58" s="12" t="str"/>
       <x:c r="M58" s="14"/>
       <x:c r="N58" s="12" t="str"/>
-      <x:c r="O58" s="4" t="str"/>
+      <x:c r="O58" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P58" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/mipi/mipi-csi-2.html</x:v>
       </x:c>
@@ -2343,7 +2461,9 @@
       <x:c r="L59" s="12" t="str"/>
       <x:c r="M59" s="14"/>
       <x:c r="N59" s="12" t="str"/>
-      <x:c r="O59" s="4" t="str"/>
+      <x:c r="O59" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P59" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/mipi/mipi-csi-2.html</x:v>
       </x:c>
@@ -2377,7 +2497,9 @@
       <x:c r="L60" s="12" t="str"/>
       <x:c r="M60" s="14"/>
       <x:c r="N60" s="12" t="str"/>
-      <x:c r="O60" s="4" t="str"/>
+      <x:c r="O60" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P60" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/mipi/d-phy.html</x:v>
       </x:c>
@@ -2411,7 +2533,9 @@
       <x:c r="L61" s="12" t="str"/>
       <x:c r="M61" s="14"/>
       <x:c r="N61" s="12" t="str"/>
-      <x:c r="O61" s="4" t="str"/>
+      <x:c r="O61" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P61" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/mipi/mipi-dsi.html</x:v>
       </x:c>
@@ -2445,7 +2569,9 @@
       <x:c r="L62" s="12" t="str"/>
       <x:c r="M62" s="14"/>
       <x:c r="N62" s="12" t="str"/>
-      <x:c r="O62" s="4" t="str"/>
+      <x:c r="O62" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P62" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/mipi/mipi-13c.html</x:v>
       </x:c>
@@ -2479,7 +2605,9 @@
       <x:c r="L63" s="12" t="str"/>
       <x:c r="M63" s="14"/>
       <x:c r="N63" s="12" t="str"/>
-      <x:c r="O63" s="4" t="str"/>
+      <x:c r="O63" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P63" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/mipi/vc-verification-ip-for-mipi-rffe.html</x:v>
       </x:c>
@@ -2513,7 +2641,9 @@
       <x:c r="L64" s="12" t="str"/>
       <x:c r="M64" s="14"/>
       <x:c r="N64" s="12" t="str"/>
-      <x:c r="O64" s="4" t="str"/>
+      <x:c r="O64" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P64" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/mipi/slimbus.html</x:v>
       </x:c>
@@ -2547,7 +2677,9 @@
       <x:c r="L65" s="12" t="str"/>
       <x:c r="M65" s="14"/>
       <x:c r="N65" s="12" t="str"/>
-      <x:c r="O65" s="4" t="str"/>
+      <x:c r="O65" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P65" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/mipi/soundwire.html</x:v>
       </x:c>
@@ -2581,7 +2713,9 @@
       <x:c r="L66" s="12" t="str"/>
       <x:c r="M66" s="14"/>
       <x:c r="N66" s="12" t="str"/>
-      <x:c r="O66" s="4" t="str"/>
+      <x:c r="O66" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P66" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/mipi/spmi.html</x:v>
       </x:c>
@@ -2615,7 +2749,9 @@
       <x:c r="L67" s="12" t="str"/>
       <x:c r="M67" s="14"/>
       <x:c r="N67" s="12" t="str"/>
-      <x:c r="O67" s="4" t="str"/>
+      <x:c r="O67" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P67" s="4" t="str">
         <x:v>https://www.synopsys.com/zh-cn/verification/verification-ip.html</x:v>
       </x:c>
@@ -2649,7 +2785,9 @@
       <x:c r="L68" s="12" t="str"/>
       <x:c r="M68" s="14"/>
       <x:c r="N68" s="12" t="str"/>
-      <x:c r="O68" s="4" t="str"/>
+      <x:c r="O68" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P68" s="4" t="str">
         <x:v>https://www.synopsys.com/zh-cn/verification/verification-ip.html</x:v>
       </x:c>
@@ -2683,7 +2821,9 @@
       <x:c r="L69" s="12" t="str"/>
       <x:c r="M69" s="14"/>
       <x:c r="N69" s="12" t="str"/>
-      <x:c r="O69" s="4" t="str"/>
+      <x:c r="O69" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P69" s="4" t="str">
         <x:v>https://www.synopsys.com/zh-cn/verification/verification-ip.html</x:v>
       </x:c>
@@ -2717,7 +2857,9 @@
       <x:c r="L70" s="12" t="str"/>
       <x:c r="M70" s="14"/>
       <x:c r="N70" s="12" t="str"/>
-      <x:c r="O70" s="4" t="str"/>
+      <x:c r="O70" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P70" s="4" t="str">
         <x:v>https://www.synopsys.com/zh-cn/verification/verification-ip.html</x:v>
       </x:c>
@@ -2751,7 +2893,9 @@
       <x:c r="L71" s="12" t="str"/>
       <x:c r="M71" s="14"/>
       <x:c r="N71" s="12" t="str"/>
-      <x:c r="O71" s="4" t="str"/>
+      <x:c r="O71" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P71" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/display/displayport.html</x:v>
       </x:c>
@@ -2785,7 +2929,9 @@
       <x:c r="L72" s="12" t="str"/>
       <x:c r="M72" s="14"/>
       <x:c r="N72" s="12" t="str"/>
-      <x:c r="O72" s="4" t="str"/>
+      <x:c r="O72" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P72" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/display/hdmi.html</x:v>
       </x:c>
@@ -2819,7 +2965,9 @@
       <x:c r="L73" s="12" t="str"/>
       <x:c r="M73" s="14"/>
       <x:c r="N73" s="12" t="str"/>
-      <x:c r="O73" s="4" t="str"/>
+      <x:c r="O73" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P73" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/12c.html</x:v>
       </x:c>
@@ -2853,7 +3001,9 @@
       <x:c r="L74" s="12" t="str"/>
       <x:c r="M74" s="14"/>
       <x:c r="N74" s="12" t="str"/>
-      <x:c r="O74" s="4" t="str"/>
+      <x:c r="O74" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P74" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/12s.html</x:v>
       </x:c>
@@ -2887,7 +3037,9 @@
       <x:c r="L75" s="12" t="str"/>
       <x:c r="M75" s="14"/>
       <x:c r="N75" s="12" t="str"/>
-      <x:c r="O75" s="4" t="str"/>
+      <x:c r="O75" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P75" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/smbus.html</x:v>
       </x:c>
@@ -2921,7 +3073,9 @@
       <x:c r="L76" s="12" t="str"/>
       <x:c r="M76" s="14"/>
       <x:c r="N76" s="12" t="str"/>
-      <x:c r="O76" s="4" t="str"/>
+      <x:c r="O76" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P76" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/uart.html</x:v>
       </x:c>
@@ -2955,7 +3109,9 @@
       <x:c r="L77" s="12" t="str"/>
       <x:c r="M77" s="14"/>
       <x:c r="N77" s="12" t="str"/>
-      <x:c r="O77" s="4" t="str"/>
+      <x:c r="O77" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P77" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/jtag.html</x:v>
       </x:c>
@@ -2989,7 +3145,9 @@
       <x:c r="L78" s="12" t="str"/>
       <x:c r="M78" s="14"/>
       <x:c r="N78" s="12" t="str"/>
-      <x:c r="O78" s="4" t="str"/>
+      <x:c r="O78" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P78" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/swd.html</x:v>
       </x:c>
@@ -3023,7 +3181,9 @@
       <x:c r="L79" s="12" t="str"/>
       <x:c r="M79" s="14"/>
       <x:c r="N79" s="12" t="str"/>
-      <x:c r="O79" s="4" t="str"/>
+      <x:c r="O79" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P79" s="4" t="str">
         <x:v>https://www.synopsys.com/blogs/chip-design/multi-domain-voltage-control-verification-avsbus-2-vip.html</x:v>
       </x:c>
@@ -3057,7 +3217,9 @@
       <x:c r="L80" s="12" t="str"/>
       <x:c r="M80" s="14"/>
       <x:c r="N80" s="12" t="str"/>
-      <x:c r="O80" s="4" t="str"/>
+      <x:c r="O80" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P80" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/sdio.html</x:v>
       </x:c>
@@ -3091,7 +3253,9 @@
       <x:c r="L81" s="12" t="str"/>
       <x:c r="M81" s="14"/>
       <x:c r="N81" s="12" t="str"/>
-      <x:c r="O81" s="4" t="str"/>
+      <x:c r="O81" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P81" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/automotive/can20-fd-tt.html</x:v>
       </x:c>
@@ -3125,7 +3289,9 @@
       <x:c r="L82" s="12" t="str"/>
       <x:c r="M82" s="14"/>
       <x:c r="N82" s="12" t="str"/>
-      <x:c r="O82" s="4" t="str"/>
+      <x:c r="O82" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P82" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/automotive/lin-verification-ip.html</x:v>
       </x:c>
@@ -3159,7 +3325,9 @@
       <x:c r="L83" s="12" t="str"/>
       <x:c r="M83" s="14"/>
       <x:c r="N83" s="12" t="str"/>
-      <x:c r="O83" s="4" t="str"/>
+      <x:c r="O83" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P83" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/automotive/flexray.html</x:v>
       </x:c>
@@ -3193,7 +3361,9 @@
       <x:c r="L84" s="12" t="str"/>
       <x:c r="M84" s="14"/>
       <x:c r="N84" s="12" t="str"/>
-      <x:c r="O84" s="4" t="str"/>
+      <x:c r="O84" s="4" t="str">
+        <x:v>Synopsys 官方</x:v>
+      </x:c>
       <x:c r="P84" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/bus-interface/vc-verification-ip-for-jesd204.html</x:v>
       </x:c>
@@ -3683,7 +3853,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40ed7c53c64a4780"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R039a294b083940ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3780,20 +3950,20 @@
       <x:c r="P4" s="1"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="15" t="str">
+      <x:c r="A5" s="21" t="str">
         <x:v>主题</x:v>
       </x:c>
-      <x:c r="B5" s="15" t="str">
+      <x:c r="B5" s="21" t="str">
         <x:v>确认问题</x:v>
       </x:c>
-      <x:c r="C5" s="15" t="str">
+      <x:c r="C5" s="21" t="str">
         <x:v>需求 / 验收依据</x:v>
       </x:c>
-      <x:c r="D5" s="15" t="str">
+      <x:c r="D5" s="21" t="str">
         <x:v>供应商答复</x:v>
       </x:c>
-      <x:c r="E5" s="1"/>
-      <x:c r="F5" s="1"/>
+      <x:c r="E5" s="22"/>
+      <x:c r="F5" s="22"/>
       <x:c r="G5" s="1"/>
       <x:c r="H5" s="1"/>
       <x:c r="I5" s="1"/>
@@ -3806,18 +3976,18 @@
       <x:c r="P5" s="1"/>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
-      <x:c r="A6" s="3" t="str">
+      <x:c r="A6" s="4" t="str">
         <x:v>商业目录</x:v>
       </x:c>
-      <x:c r="B6" s="3" t="str">
+      <x:c r="B6" s="4" t="str">
         <x:v>请提供当前完整VIP SKU及bundle清单</x:v>
       </x:c>
-      <x:c r="C6" s="3" t="str">
+      <x:c r="C6" s="4" t="str">
         <x:v>将本表每一行映射至SKU、License Feature及包内范围，补充未列出的可售产品。</x:v>
       </x:c>
-      <x:c r="D6" s="16" t="str"/>
-      <x:c r="E6" s="1"/>
-      <x:c r="F6" s="1"/>
+      <x:c r="D6" s="12" t="str"/>
+      <x:c r="E6" s="22"/>
+      <x:c r="F6" s="22"/>
       <x:c r="G6" s="1"/>
       <x:c r="H6" s="1"/>
       <x:c r="I6" s="1"/>
@@ -3830,18 +4000,18 @@
       <x:c r="P6" s="1"/>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
-      <x:c r="A7" s="3" t="str">
+      <x:c r="A7" s="4" t="str">
         <x:v>协议版本</x:v>
       </x:c>
-      <x:c r="B7" s="3" t="str">
+      <x:c r="B7" s="4" t="str">
         <x:v>精确规范与release矩阵是什么？</x:v>
       </x:c>
-      <x:c r="C7" s="3" t="str">
+      <x:c r="C7" s="4" t="str">
         <x:v>区分正式标准、draft、预览和研发路线图，列出已支持/未支持特性。</x:v>
       </x:c>
-      <x:c r="D7" s="16" t="str"/>
-      <x:c r="E7" s="1"/>
-      <x:c r="F7" s="1"/>
+      <x:c r="D7" s="12" t="str"/>
+      <x:c r="E7" s="22"/>
+      <x:c r="F7" s="22"/>
       <x:c r="G7" s="1"/>
       <x:c r="H7" s="1"/>
       <x:c r="I7" s="1"/>
@@ -3854,18 +4024,18 @@
       <x:c r="P7" s="1"/>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
-      <x:c r="A8" s="3" t="str">
+      <x:c r="A8" s="4" t="str">
         <x:v>角色与层次</x:v>
       </x:c>
-      <x:c r="B8" s="3" t="str">
+      <x:c r="B8" s="4" t="str">
         <x:v>每个VIP包含哪些角色和接口层？</x:v>
       </x:c>
-      <x:c r="C8" s="3" t="str">
+      <x:c r="C8" s="4" t="str">
         <x:v>确认master/slave/monitor，host/device，serial/PIPE/PPI/transaction-level及错误注入。</x:v>
       </x:c>
-      <x:c r="D8" s="16" t="str"/>
-      <x:c r="E8" s="1"/>
-      <x:c r="F8" s="1"/>
+      <x:c r="D8" s="12" t="str"/>
+      <x:c r="E8" s="22"/>
+      <x:c r="F8" s="22"/>
       <x:c r="G8" s="1"/>
       <x:c r="H8" s="1"/>
       <x:c r="I8" s="1"/>
@@ -3878,18 +4048,18 @@
       <x:c r="P8" s="1"/>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
-      <x:c r="A9" s="3" t="str">
+      <x:c r="A9" s="4" t="str">
         <x:v>依赖与重叠</x:v>
       </x:c>
-      <x:c r="B9" s="3" t="str">
+      <x:c r="B9" s="4" t="str">
         <x:v>哪些需要额外VIP或选件？</x:v>
       </x:c>
-      <x:c r="C9" s="3" t="str">
+      <x:c r="C9" s="4" t="str">
         <x:v>特别是CHI C2C→CHI，UFS→UniPro/M-PHY，USB4隧道，以及SD/UHS-II/eMMC、SPI各形态去重。</x:v>
       </x:c>
-      <x:c r="D9" s="16" t="str"/>
-      <x:c r="E9" s="1"/>
-      <x:c r="F9" s="1"/>
+      <x:c r="D9" s="12" t="str"/>
+      <x:c r="E9" s="22"/>
+      <x:c r="F9" s="22"/>
       <x:c r="G9" s="1"/>
       <x:c r="H9" s="1"/>
       <x:c r="I9" s="1"/>
@@ -3902,18 +4072,18 @@
       <x:c r="P9" s="1"/>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
-      <x:c r="A10" s="3" t="str">
+      <x:c r="A10" s="4" t="str">
         <x:v>仿真器兼容</x:v>
       </x:c>
-      <x:c r="B10" s="3" t="str">
+      <x:c r="B10" s="4" t="str">
         <x:v>VCS、Xcelium和UVM1.2精确组合支持？</x:v>
       </x:c>
-      <x:c r="C10" s="3" t="str">
+      <x:c r="C10" s="4" t="str">
         <x:v>要求双方约定版本的release matrix及可执行示例。不要只写“支持主流仿真器”。</x:v>
       </x:c>
-      <x:c r="D10" s="16" t="str"/>
-      <x:c r="E10" s="1"/>
-      <x:c r="F10" s="1"/>
+      <x:c r="D10" s="12" t="str"/>
+      <x:c r="E10" s="22"/>
+      <x:c r="F10" s="22"/>
       <x:c r="G10" s="1"/>
       <x:c r="H10" s="1"/>
       <x:c r="I10" s="1"/>
@@ -3926,18 +4096,18 @@
       <x:c r="P10" s="1"/>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
-      <x:c r="A11" s="3" t="str">
+      <x:c r="A11" s="4" t="str">
         <x:v>服务器环境</x:v>
       </x:c>
-      <x:c r="B11" s="3" t="str">
+      <x:c r="B11" s="4" t="str">
         <x:v>当前Linux发行版和glibc是否支持？</x:v>
       </x:c>
-      <x:c r="C11" s="3" t="str">
+      <x:c r="C11" s="4" t="str">
         <x:v>确认编译器、DPI库、位宽、依赖、安装权限及离线部署流程。</x:v>
       </x:c>
-      <x:c r="D11" s="16" t="str"/>
-      <x:c r="E11" s="1"/>
-      <x:c r="F11" s="1"/>
+      <x:c r="D11" s="12" t="str"/>
+      <x:c r="E11" s="22"/>
+      <x:c r="F11" s="22"/>
       <x:c r="G11" s="1"/>
       <x:c r="H11" s="1"/>
       <x:c r="I11" s="1"/>
@@ -3950,18 +4120,18 @@
       <x:c r="P11" s="1"/>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
-      <x:c r="A12" s="3" t="str">
+      <x:c r="A12" s="4" t="str">
         <x:v>并行回归</x:v>
       </x:c>
-      <x:c r="B12" s="3" t="str">
+      <x:c r="B12" s="4" t="str">
         <x:v>LSF回归怎样消耗license？</x:v>
       </x:c>
-      <x:c r="C12" s="3" t="str">
+      <x:c r="C12" s="4" t="str">
         <x:v>按仿真进程、实例、协议、端口还是token？同一test多个VIP消耗多少？给出并发例子。</x:v>
       </x:c>
-      <x:c r="D12" s="16" t="str"/>
-      <x:c r="E12" s="1"/>
-      <x:c r="F12" s="1"/>
+      <x:c r="D12" s="12" t="str"/>
+      <x:c r="E12" s="22"/>
+      <x:c r="F12" s="22"/>
       <x:c r="G12" s="1"/>
       <x:c r="H12" s="1"/>
       <x:c r="I12" s="1"/>
@@ -3974,18 +4144,18 @@
       <x:c r="P12" s="1"/>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
-      <x:c r="A13" s="3" t="str">
+      <x:c r="A13" s="4" t="str">
         <x:v>授权范围</x:v>
       </x:c>
-      <x:c r="B13" s="3" t="str">
+      <x:c r="B13" s="4" t="str">
         <x:v>授权期限、地域和项目范围是什么？</x:v>
       </x:c>
-      <x:c r="C13" s="3" t="str">
+      <x:c r="C13" s="4" t="str">
         <x:v>确认浮动池、跨服务器/站点、多项目复用、续费及版本升级权益。</x:v>
       </x:c>
-      <x:c r="D13" s="16" t="str"/>
-      <x:c r="E13" s="1"/>
-      <x:c r="F13" s="1"/>
+      <x:c r="D13" s="12" t="str"/>
+      <x:c r="E13" s="22"/>
+      <x:c r="F13" s="22"/>
       <x:c r="G13" s="1"/>
       <x:c r="H13" s="1"/>
       <x:c r="I13" s="1"/>
@@ -3998,18 +4168,18 @@
       <x:c r="P13" s="1"/>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
-      <x:c r="A14" s="3" t="str">
+      <x:c r="A14" s="4" t="str">
         <x:v>测试套件</x:v>
       </x:c>
-      <x:c r="B14" s="3" t="str">
+      <x:c r="B14" s="4" t="str">
         <x:v>Test Suite和验证计划是否包含？</x:v>
       </x:c>
-      <x:c r="C14" s="3" t="str">
+      <x:c r="C14" s="4" t="str">
         <x:v>逐协议确认源码用例、可修改权、coverage plan、错误场景及是否独立收费。</x:v>
       </x:c>
-      <x:c r="D14" s="16" t="str"/>
-      <x:c r="E14" s="1"/>
-      <x:c r="F14" s="1"/>
+      <x:c r="D14" s="12" t="str"/>
+      <x:c r="E14" s="22"/>
+      <x:c r="F14" s="22"/>
       <x:c r="G14" s="1"/>
       <x:c r="H14" s="1"/>
       <x:c r="I14" s="1"/>
@@ -4022,18 +4192,18 @@
       <x:c r="P14" s="1"/>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
-      <x:c r="A15" s="3" t="str">
+      <x:c r="A15" s="4" t="str">
         <x:v>系统检查</x:v>
       </x:c>
-      <x:c r="B15" s="3" t="str">
+      <x:c r="B15" s="4" t="str">
         <x:v>系统一致性、数据检查和性能组件是否包含？</x:v>
       </x:c>
-      <x:c r="C15" s="3" t="str">
+      <x:c r="C15" s="4" t="str">
         <x:v>核对interconnect model、system monitor、scoreboard、traffic profile及调试工具依赖。</x:v>
       </x:c>
-      <x:c r="D15" s="16" t="str"/>
-      <x:c r="E15" s="1"/>
-      <x:c r="F15" s="1"/>
+      <x:c r="D15" s="12" t="str"/>
+      <x:c r="E15" s="22"/>
+      <x:c r="F15" s="22"/>
       <x:c r="G15" s="1"/>
       <x:c r="H15" s="1"/>
       <x:c r="I15" s="1"/>
@@ -4046,18 +4216,18 @@
       <x:c r="P15" s="1"/>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
-      <x:c r="A16" s="3" t="str">
+      <x:c r="A16" s="4" t="str">
         <x:v>初期DDR替代</x:v>
       </x:c>
-      <x:c r="B16" s="3" t="str">
+      <x:c r="B16" s="4" t="str">
         <x:v>AXI slave memory responder能否满足冒烟？</x:v>
       </x:c>
-      <x:c r="C16" s="3" t="str">
+      <x:c r="C16" s="4" t="str">
         <x:v>需要镜像预装载、读写backdoor、字节使能、burst/ID/outstanding、错误和延迟可控。</x:v>
       </x:c>
-      <x:c r="D16" s="16" t="str"/>
-      <x:c r="E16" s="1"/>
-      <x:c r="F16" s="1"/>
+      <x:c r="D16" s="12" t="str"/>
+      <x:c r="E16" s="22"/>
+      <x:c r="F16" s="22"/>
       <x:c r="G16" s="1"/>
       <x:c r="H16" s="1"/>
       <x:c r="I16" s="1"/>
@@ -4070,18 +4240,18 @@
       <x:c r="P16" s="1"/>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
-      <x:c r="A17" s="3" t="str">
+      <x:c r="A17" s="4" t="str">
         <x:v>真实内存</x:v>
       </x:c>
-      <x:c r="B17" s="3" t="str">
+      <x:c r="B17" s="4" t="str">
         <x:v>DDR/DFI/颗粒模型覆盖哪些边界？</x:v>
       </x:c>
-      <x:c r="C17" s="3" t="str">
+      <x:c r="C17" s="4" t="str">
         <x:v>列器件型号、rank/DIMM、training、低功耗和时序检查；不把AXI memory responder当DDR验证。</x:v>
       </x:c>
-      <x:c r="D17" s="16" t="str"/>
-      <x:c r="E17" s="1"/>
-      <x:c r="F17" s="1"/>
+      <x:c r="D17" s="12" t="str"/>
+      <x:c r="E17" s="22"/>
+      <x:c r="F17" s="22"/>
       <x:c r="G17" s="1"/>
       <x:c r="H17" s="1"/>
       <x:c r="I17" s="1"/>
@@ -4094,18 +4264,18 @@
       <x:c r="P17" s="1"/>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
-      <x:c r="A18" s="3" t="str">
+      <x:c r="A18" s="4" t="str">
         <x:v>硬件辅助验证</x:v>
       </x:c>
-      <x:c r="B18" s="3" t="str">
+      <x:c r="B18" s="4" t="str">
         <x:v>RTL仿真与ZeBu/Palladium支持如何划分？</x:v>
       </x:c>
-      <x:c r="C18" s="3" t="str">
+      <x:c r="C18" s="4" t="str">
         <x:v>单独确认transactor/加速方案、平台版本、可综合部分和授权，不能由SV VIP推断可用。</x:v>
       </x:c>
-      <x:c r="D18" s="16" t="str"/>
-      <x:c r="E18" s="1"/>
-      <x:c r="F18" s="1"/>
+      <x:c r="D18" s="12" t="str"/>
+      <x:c r="E18" s="22"/>
+      <x:c r="F18" s="22"/>
       <x:c r="G18" s="1"/>
       <x:c r="H18" s="1"/>
       <x:c r="I18" s="1"/>
@@ -4118,18 +4288,18 @@
       <x:c r="P18" s="1"/>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
-      <x:c r="A19" s="3" t="str">
+      <x:c r="A19" s="4" t="str">
         <x:v>交付验收</x:v>
       </x:c>
-      <x:c r="B19" s="3" t="str">
+      <x:c r="B19" s="4" t="str">
         <x:v>可否用双方仿真器跑采购验收list？</x:v>
       </x:c>
-      <x:c r="C19" s="3" t="str">
+      <x:c r="C19" s="4" t="str">
         <x:v>包含正常/异常、reset、中断/低功耗（适用时）、coverage、monitor与预期失败检查。</x:v>
       </x:c>
-      <x:c r="D19" s="16" t="str"/>
-      <x:c r="E19" s="1"/>
-      <x:c r="F19" s="1"/>
+      <x:c r="D19" s="12" t="str"/>
+      <x:c r="E19" s="22"/>
+      <x:c r="F19" s="22"/>
       <x:c r="G19" s="1"/>
       <x:c r="H19" s="1"/>
       <x:c r="I19" s="1"/>
@@ -4142,18 +4312,18 @@
       <x:c r="P19" s="1"/>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
-      <x:c r="A20" s="3" t="str">
+      <x:c r="A20" s="4" t="str">
         <x:v>维护服务</x:v>
       </x:c>
-      <x:c r="B20" s="3" t="str">
+      <x:c r="B20" s="4" t="str">
         <x:v>维护、升级及问题响应约定？</x:v>
       </x:c>
-      <x:c r="C20" s="3" t="str">
+      <x:c r="C20" s="4" t="str">
         <x:v>确认FAE支持、缺陷修复、版本升级、文档培训和交付时间。</x:v>
       </x:c>
-      <x:c r="D20" s="16" t="str"/>
-      <x:c r="E20" s="1"/>
-      <x:c r="F20" s="1"/>
+      <x:c r="D20" s="12" t="str"/>
+      <x:c r="E20" s="22"/>
+      <x:c r="F20" s="22"/>
       <x:c r="G20" s="1"/>
       <x:c r="H20" s="1"/>
       <x:c r="I20" s="1"/>
@@ -4166,18 +4336,18 @@
       <x:c r="P20" s="1"/>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
-      <x:c r="A21" s="3" t="str">
+      <x:c r="A21" s="4" t="str">
         <x:v>报价</x:v>
       </x:c>
-      <x:c r="B21" s="3" t="str">
+      <x:c r="B21" s="4" t="str">
         <x:v>请逐项或bundle报价并列商业条件</x:v>
       </x:c>
-      <x:c r="C21" s="3" t="str">
+      <x:c r="C21" s="4" t="str">
         <x:v>填写SKU、Feature、并发数、币种、税、维护期、折扣基础及报价有效期，避免重复采购。</x:v>
       </x:c>
-      <x:c r="D21" s="16" t="str"/>
-      <x:c r="E21" s="1"/>
-      <x:c r="F21" s="1"/>
+      <x:c r="D21" s="12" t="str"/>
+      <x:c r="E21" s="22"/>
+      <x:c r="F21" s="22"/>
       <x:c r="G21" s="1"/>
       <x:c r="H21" s="1"/>
       <x:c r="I21" s="1"/>
@@ -4190,12 +4360,12 @@
       <x:c r="P21" s="1"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="1"/>
-      <x:c r="B22" s="1"/>
-      <x:c r="C22" s="1"/>
-      <x:c r="D22" s="1"/>
-      <x:c r="E22" s="1"/>
-      <x:c r="F22" s="1"/>
+      <x:c r="A22" s="22"/>
+      <x:c r="B22" s="22"/>
+      <x:c r="C22" s="22"/>
+      <x:c r="D22" s="22"/>
+      <x:c r="E22" s="22"/>
+      <x:c r="F22" s="22"/>
       <x:c r="G22" s="1"/>
       <x:c r="H22" s="1"/>
       <x:c r="I22" s="1"/>
@@ -4208,12 +4378,12 @@
       <x:c r="P22" s="1"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="1"/>
-      <x:c r="B23" s="1"/>
-      <x:c r="C23" s="1"/>
-      <x:c r="D23" s="1"/>
-      <x:c r="E23" s="1"/>
-      <x:c r="F23" s="1"/>
+      <x:c r="A23" s="22"/>
+      <x:c r="B23" s="22"/>
+      <x:c r="C23" s="22"/>
+      <x:c r="D23" s="22"/>
+      <x:c r="E23" s="22"/>
+      <x:c r="F23" s="22"/>
       <x:c r="G23" s="1"/>
       <x:c r="H23" s="1"/>
       <x:c r="I23" s="1"/>
@@ -4226,14 +4396,14 @@
       <x:c r="P23" s="1"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="17" t="str">
+      <x:c r="A24" s="23" t="str">
         <x:v>待核实项目、配套方案与补充证据</x:v>
       </x:c>
-      <x:c r="B24" s="1"/>
-      <x:c r="C24" s="1"/>
-      <x:c r="D24" s="1"/>
-      <x:c r="E24" s="1"/>
-      <x:c r="F24" s="1"/>
+      <x:c r="B24" s="22"/>
+      <x:c r="C24" s="22"/>
+      <x:c r="D24" s="22"/>
+      <x:c r="E24" s="22"/>
+      <x:c r="F24" s="22"/>
       <x:c r="G24" s="1"/>
       <x:c r="H24" s="1"/>
       <x:c r="I24" s="1"/>
@@ -4246,12 +4416,12 @@
       <x:c r="P24" s="1"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="1"/>
-      <x:c r="B25" s="1"/>
-      <x:c r="C25" s="1"/>
-      <x:c r="D25" s="1"/>
-      <x:c r="E25" s="1"/>
-      <x:c r="F25" s="1"/>
+      <x:c r="A25" s="22"/>
+      <x:c r="B25" s="22"/>
+      <x:c r="C25" s="22"/>
+      <x:c r="D25" s="22"/>
+      <x:c r="E25" s="22"/>
+      <x:c r="F25" s="22"/>
       <x:c r="G25" s="1"/>
       <x:c r="H25" s="1"/>
       <x:c r="I25" s="1"/>
@@ -4264,20 +4434,20 @@
       <x:c r="P25" s="1"/>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
-      <x:c r="A26" s="20" t="str">
+      <x:c r="A26" s="24" t="str">
         <x:v>类型</x:v>
       </x:c>
-      <x:c r="B26" s="20" t="str">
+      <x:c r="B26" s="24" t="str">
         <x:v>项目</x:v>
       </x:c>
-      <x:c r="C26" s="20" t="str">
+      <x:c r="C26" s="24" t="str">
         <x:v>当前证据 / 待确认范围</x:v>
       </x:c>
-      <x:c r="D26" s="20" t="str">
+      <x:c r="D26" s="24" t="str">
         <x:v>供应商答复</x:v>
       </x:c>
-      <x:c r="E26" s="1" t="str"/>
-      <x:c r="F26" s="1" t="str">
+      <x:c r="E26" s="22" t="str"/>
+      <x:c r="F26" s="22" t="str">
         <x:v>官方来源 URL</x:v>
       </x:c>
       <x:c r="G26" s="1"/>
@@ -4292,18 +4462,18 @@
       <x:c r="P26" s="1"/>
     </x:row>
     <x:row r="27" ht="62" customHeight="1">
-      <x:c r="A27" s="3" t="str">
+      <x:c r="A27" s="4" t="str">
         <x:v>待核实产品</x:v>
       </x:c>
-      <x:c r="B27" s="3" t="str">
+      <x:c r="B27" s="4" t="str">
         <x:v>CAN XL</x:v>
       </x:c>
-      <x:c r="C27" s="3" t="str">
+      <x:c r="C27" s="4" t="str">
         <x:v>现有CAN2.0/FD/TT不能证明CAN XL支持；请提供官方产品与release信息。</x:v>
       </x:c>
-      <x:c r="D27" s="16" t="str"/>
-      <x:c r="E27" s="3" t="str"/>
-      <x:c r="F27" s="3" t="str"/>
+      <x:c r="D27" s="12" t="str"/>
+      <x:c r="E27" s="4" t="str"/>
+      <x:c r="F27" s="4" t="str"/>
       <x:c r="G27" s="1"/>
       <x:c r="H27" s="1"/>
       <x:c r="I27" s="1"/>
@@ -4316,18 +4486,18 @@
       <x:c r="P27" s="1"/>
     </x:row>
     <x:row r="28" ht="62" customHeight="1">
-      <x:c r="A28" s="3" t="str">
+      <x:c r="A28" s="4" t="str">
         <x:v>待核实产品</x:v>
       </x:c>
-      <x:c r="B28" s="3" t="str">
+      <x:c r="B28" s="4" t="str">
         <x:v>完整PMBus / MCTP</x:v>
       </x:c>
-      <x:c r="C28" s="3" t="str">
+      <x:c r="C28" s="4" t="str">
         <x:v>AVSBus不等于PMBus Part I/II或MCTP；服务器管理场景单独询价。</x:v>
       </x:c>
-      <x:c r="D28" s="16" t="str"/>
-      <x:c r="E28" s="3" t="str"/>
-      <x:c r="F28" s="3" t="str"/>
+      <x:c r="D28" s="12" t="str"/>
+      <x:c r="E28" s="4" t="str"/>
+      <x:c r="F28" s="4" t="str"/>
       <x:c r="G28" s="1"/>
       <x:c r="H28" s="1"/>
       <x:c r="I28" s="1"/>
@@ -4340,18 +4510,18 @@
       <x:c r="P28" s="1"/>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
-      <x:c r="A29" s="3" t="str">
+      <x:c r="A29" s="4" t="str">
         <x:v>待核实产品</x:v>
       </x:c>
-      <x:c r="B29" s="3" t="str">
+      <x:c r="B29" s="4" t="str">
         <x:v>eSPI / LPC</x:v>
       </x:c>
-      <x:c r="C29" s="3" t="str">
+      <x:c r="C29" s="4" t="str">
         <x:v>本次未取得足够官方VIP证据，不代表不存在。</x:v>
       </x:c>
-      <x:c r="D29" s="16" t="str"/>
-      <x:c r="E29" s="3" t="str"/>
-      <x:c r="F29" s="3" t="str"/>
+      <x:c r="D29" s="12" t="str"/>
+      <x:c r="E29" s="4" t="str"/>
+      <x:c r="F29" s="4" t="str"/>
       <x:c r="G29" s="1"/>
       <x:c r="H29" s="1"/>
       <x:c r="I29" s="1"/>
@@ -4364,18 +4534,18 @@
       <x:c r="P29" s="1"/>
     </x:row>
     <x:row r="30" ht="62" customHeight="1">
-      <x:c r="A30" s="3" t="str">
+      <x:c r="A30" s="4" t="str">
         <x:v>待核实产品</x:v>
       </x:c>
-      <x:c r="B30" s="3" t="str">
+      <x:c r="B30" s="4" t="str">
         <x:v>RoCE / InfiniBand</x:v>
       </x:c>
-      <x:c r="C30" s="3" t="str">
+      <x:c r="C30" s="4" t="str">
         <x:v>不从Ethernet或Ultra Ethernet支持推断完整协议VIP。</x:v>
       </x:c>
-      <x:c r="D30" s="16" t="str"/>
-      <x:c r="E30" s="3" t="str"/>
-      <x:c r="F30" s="3" t="str"/>
+      <x:c r="D30" s="12" t="str"/>
+      <x:c r="E30" s="4" t="str"/>
+      <x:c r="F30" s="4" t="str"/>
       <x:c r="G30" s="1"/>
       <x:c r="H30" s="1"/>
       <x:c r="I30" s="1"/>
@@ -4388,18 +4558,18 @@
       <x:c r="P30" s="1"/>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
-      <x:c r="A31" s="3" t="str">
+      <x:c r="A31" s="4" t="str">
         <x:v>待核实产品</x:v>
       </x:c>
-      <x:c r="B31" s="3" t="str">
+      <x:c r="B31" s="4" t="str">
         <x:v>MIPI A-PHY</x:v>
       </x:c>
-      <x:c r="C31" s="3" t="str">
+      <x:c r="C31" s="4" t="str">
         <x:v>不能从C-PHY/D-PHY产品推断。</x:v>
       </x:c>
-      <x:c r="D31" s="16" t="str"/>
-      <x:c r="E31" s="3" t="str"/>
-      <x:c r="F31" s="3" t="str"/>
+      <x:c r="D31" s="12" t="str"/>
+      <x:c r="E31" s="4" t="str"/>
+      <x:c r="F31" s="4" t="str"/>
       <x:c r="G31" s="1"/>
       <x:c r="H31" s="1"/>
       <x:c r="I31" s="1"/>
@@ -4412,18 +4582,18 @@
       <x:c r="P31" s="1"/>
     </x:row>
     <x:row r="32" ht="62" customHeight="1">
-      <x:c r="A32" s="3" t="str">
+      <x:c r="A32" s="4" t="str">
         <x:v>待核实产品</x:v>
       </x:c>
-      <x:c r="B32" s="3" t="str">
+      <x:c r="B32" s="4" t="str">
         <x:v>GDDR7</x:v>
       </x:c>
-      <x:c r="C32" s="3" t="str">
+      <x:c r="C32" s="4" t="str">
         <x:v>本次未核实可交付release和SKU，应由销售说明现有版本或路线图。</x:v>
       </x:c>
-      <x:c r="D32" s="16" t="str"/>
-      <x:c r="E32" s="3" t="str"/>
-      <x:c r="F32" s="3" t="str"/>
+      <x:c r="D32" s="12" t="str"/>
+      <x:c r="E32" s="4" t="str"/>
+      <x:c r="F32" s="4" t="str"/>
       <x:c r="G32" s="1"/>
       <x:c r="H32" s="1"/>
       <x:c r="I32" s="1"/>
@@ -4436,18 +4606,18 @@
       <x:c r="P32" s="1"/>
     </x:row>
     <x:row r="33" ht="62" customHeight="1">
-      <x:c r="A33" s="3" t="str">
+      <x:c r="A33" s="4" t="str">
         <x:v>官方公告线索</x:v>
       </x:c>
-      <x:c r="B33" s="3" t="str">
+      <x:c r="B33" s="4" t="str">
         <x:v>DDR6</x:v>
       </x:c>
-      <x:c r="C33" s="3" t="str">
+      <x:c r="C33" s="4" t="str">
         <x:v>官方作者页已有2026-08-14介绍文章；交付release及GA状态待销售确认。</x:v>
       </x:c>
-      <x:c r="D33" s="16" t="str"/>
-      <x:c r="E33" s="3" t="str"/>
-      <x:c r="F33" s="3" t="str">
+      <x:c r="D33" s="12" t="str"/>
+      <x:c r="E33" s="4" t="str"/>
+      <x:c r="F33" s="4" t="str">
         <x:v>https://www.synopsys.com/authors/gaurav-kumar.html</x:v>
       </x:c>
       <x:c r="G33" s="1"/>
@@ -4462,18 +4632,18 @@
       <x:c r="P33" s="1"/>
     </x:row>
     <x:row r="34" ht="62" customHeight="1">
-      <x:c r="A34" s="3" t="str">
+      <x:c r="A34" s="4" t="str">
         <x:v>研发路线图</x:v>
       </x:c>
-      <x:c r="B34" s="3" t="str">
+      <x:c r="B34" s="4" t="str">
         <x:v>HBM5</x:v>
       </x:c>
-      <x:c r="C34" s="3" t="str">
+      <x:c r="C34" s="4" t="str">
         <x:v>官方文章表述正在开发，JEDEC Draft1.0-04；不能列作已确认可售交付。</x:v>
       </x:c>
-      <x:c r="D34" s="16" t="str"/>
-      <x:c r="E34" s="3" t="str"/>
-      <x:c r="F34" s="3" t="str">
+      <x:c r="D34" s="12" t="str"/>
+      <x:c r="E34" s="4" t="str"/>
+      <x:c r="F34" s="4" t="str">
         <x:v>https://www.synopsys.com/blogs/chip-design/ai-accelerators-hbm5-verification-ip.html</x:v>
       </x:c>
       <x:c r="G34" s="1"/>
@@ -4488,18 +4658,18 @@
       <x:c r="P34" s="1"/>
     </x:row>
     <x:row r="35" ht="62" customHeight="1">
-      <x:c r="A35" s="3" t="str">
+      <x:c r="A35" s="4" t="str">
         <x:v>配套方案</x:v>
       </x:c>
-      <x:c r="B35" s="3" t="str">
+      <x:c r="B35" s="4" t="str">
         <x:v>Synopsys Test Suites</x:v>
       </x:c>
-      <x:c r="C35" s="3" t="str">
+      <x:c r="C35" s="4" t="str">
         <x:v>按协议确认是否含源码、是否另售；AMBA与其它协议可能不同。</x:v>
       </x:c>
-      <x:c r="D35" s="16" t="str"/>
-      <x:c r="E35" s="3" t="str"/>
-      <x:c r="F35" s="3" t="str">
+      <x:c r="D35" s="12" t="str"/>
+      <x:c r="E35" s="4" t="str"/>
+      <x:c r="F35" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/verification-test-suites.html</x:v>
       </x:c>
       <x:c r="G35" s="1"/>
@@ -4514,18 +4684,18 @@
       <x:c r="P35" s="1"/>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
-      <x:c r="A36" s="3" t="str">
+      <x:c r="A36" s="4" t="str">
         <x:v>配套方案</x:v>
       </x:c>
-      <x:c r="B36" s="3" t="str">
+      <x:c r="B36" s="4" t="str">
         <x:v>UNH Ethernet Test Suites</x:v>
       </x:c>
-      <x:c r="C36" s="3" t="str">
+      <x:c r="C36" s="4" t="str">
         <x:v>官方目录列出，需确认当前提供方式及许可。</x:v>
       </x:c>
-      <x:c r="D36" s="16" t="str"/>
-      <x:c r="E36" s="3" t="str"/>
-      <x:c r="F36" s="3" t="str">
+      <x:c r="D36" s="12" t="str"/>
+      <x:c r="E36" s="4" t="str"/>
+      <x:c r="F36" s="4" t="str">
         <x:v>https://www.synopsys.com/zh-cn/verification/verification-ip.html</x:v>
       </x:c>
       <x:c r="G36" s="1"/>
@@ -4540,18 +4710,18 @@
       <x:c r="P36" s="1"/>
     </x:row>
     <x:row r="37" ht="62" customHeight="1">
-      <x:c r="A37" s="3" t="str">
+      <x:c r="A37" s="4" t="str">
         <x:v>配套方案</x:v>
       </x:c>
-      <x:c r="B37" s="3" t="str">
+      <x:c r="B37" s="4" t="str">
         <x:v>VC SoC AutoTestbench / AutoPerformance</x:v>
       </x:c>
-      <x:c r="C37" s="3" t="str">
+      <x:c r="C37" s="4" t="str">
         <x:v>环境生成与性能方案，单独询价，不计作独立协议VIP。</x:v>
       </x:c>
-      <x:c r="D37" s="16" t="str"/>
-      <x:c r="E37" s="3" t="str"/>
-      <x:c r="F37" s="3" t="str">
+      <x:c r="D37" s="12" t="str"/>
+      <x:c r="E37" s="4" t="str"/>
+      <x:c r="F37" s="4" t="str">
         <x:v>https://www.synopsys.com/verification/verification-ip/amba.html</x:v>
       </x:c>
       <x:c r="G37" s="1"/>
@@ -4566,18 +4736,18 @@
       <x:c r="P37" s="1"/>
     </x:row>
     <x:row r="38" ht="62" customHeight="1">
-      <x:c r="A38" s="3" t="str">
+      <x:c r="A38" s="4" t="str">
         <x:v>补充版本证据</x:v>
       </x:c>
-      <x:c r="B38" s="3" t="str">
+      <x:c r="B38" s="4" t="str">
         <x:v>PCIe8 Draft0.3</x:v>
       </x:c>
-      <x:c r="C38" s="3" t="str">
+      <x:c r="C38" s="4" t="str">
         <x:v>官方博客确认草案支持；要求销售对照交付release确认。</x:v>
       </x:c>
-      <x:c r="D38" s="16" t="str"/>
-      <x:c r="E38" s="3" t="str"/>
-      <x:c r="F38" s="3" t="str">
+      <x:c r="D38" s="12" t="str"/>
+      <x:c r="E38" s="4" t="str"/>
+      <x:c r="F38" s="4" t="str">
         <x:v>https://www.synopsys.com/blogs/chip-design/pcie-8-0-verification-ip-ai-hpc-automotive.html</x:v>
       </x:c>
       <x:c r="G38" s="1"/>
@@ -4592,18 +4762,18 @@
       <x:c r="P38" s="1"/>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
-      <x:c r="A39" s="3" t="str">
+      <x:c r="A39" s="4" t="str">
         <x:v>补充功能证据</x:v>
       </x:c>
-      <x:c r="B39" s="3" t="str">
+      <x:c r="B39" s="4" t="str">
         <x:v>MIPI CSE2.0</x:v>
       </x:c>
-      <x:c r="C39" s="3" t="str">
+      <x:c r="C39" s="4" t="str">
         <x:v>CSI-2安全扩展需求，不能直接推断独立SKU。</x:v>
       </x:c>
-      <x:c r="D39" s="16" t="str"/>
-      <x:c r="E39" s="3" t="str"/>
-      <x:c r="F39" s="3" t="str">
+      <x:c r="D39" s="12" t="str"/>
+      <x:c r="E39" s="4" t="str"/>
+      <x:c r="F39" s="4" t="str">
         <x:v>https://www.synopsys.com/blogs/chip-design/streamlining-camera-security-validation-framework-using-synopsys-mipi-cse-v20-vip.html</x:v>
       </x:c>
       <x:c r="G39" s="1"/>
@@ -4618,18 +4788,18 @@
       <x:c r="P39" s="1"/>
     </x:row>
     <x:row r="40" ht="62" customHeight="1">
-      <x:c r="A40" s="3" t="str">
+      <x:c r="A40" s="4" t="str">
         <x:v>补充功能证据</x:v>
       </x:c>
-      <x:c r="B40" s="3" t="str">
+      <x:c r="B40" s="4" t="str">
         <x:v>I3C HDR multi-lane</x:v>
       </x:c>
-      <x:c r="C40" s="3" t="str">
+      <x:c r="C40" s="4" t="str">
         <x:v>官方博客有覆盖说明；具体规范revision请销售确认。</x:v>
       </x:c>
-      <x:c r="D40" s="16" t="str"/>
-      <x:c r="E40" s="3" t="str"/>
-      <x:c r="F40" s="3" t="str">
+      <x:c r="D40" s="12" t="str"/>
+      <x:c r="E40" s="4" t="str"/>
+      <x:c r="F40" s="4" t="str">
         <x:v>https://www.synopsys.com/blogs/chip-design/i3c-vip-hdr-multi-lane-verification.html</x:v>
       </x:c>
       <x:c r="G40" s="1"/>
@@ -5906,8 +6076,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8aa36621a4dd467b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd0c0a1c06746cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11b28ea8212b45a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93a499d669cb4285"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>